<commit_message>
Tennis Fanrecap: Full pipeline run 2026-04-22
5 stories: Fils wins Barcelona (4th title, injury comeback); Shelton wins Munich
(first American since Agassi 2002 to win ATP 500+ clay); Rybakina wins Stuttgart
(13th title, first repeat); Alcaraz arm cast/French Open doubt; Madrid Open opens.

9 X posts, 5 FB posts, 5 articles, PostPlanner exports (standard + TOBI).

https://claude.ai/code/session_01JnnE96thfGL1xc4nGLpTtk
</commit_message>
<xml_diff>
--- a/Tennis/postplanner-imports/tfr-postplanner-2026-04-18.xlsx
+++ b/Tennis/postplanner-imports/tfr-postplanner-2026-04-18.xlsx
@@ -478,7 +478,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>04/18/2026  12:56</t>
+          <t>04/18/2026  08:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -493,7 +493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>04/18/2026  14:13</t>
+          <t>04/18/2026  10:30</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -508,7 +508,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>04/18/2026  15:30</t>
+          <t>04/18/2026  12:30</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -522,7 +522,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04/18/2026  16:47</t>
+          <t>04/18/2026  15:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04/18/2026  18:04</t>
+          <t>04/18/2026  18:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -550,7 +550,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04/18/2026  19:21</t>
+          <t>04/18/2026  21:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -564,7 +564,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04/18/2026  20:38</t>
+          <t>04/18/2026  21:05</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">

</xml_diff>